<commit_message>
Auto-deploy updates: Tue 09/29/2026 12:55:56.27
</commit_message>
<xml_diff>
--- a/NEET_2026_Targets_Template.xlsx
+++ b/NEET_2026_Targets_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Projects\NEET Analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\NEET Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C610CABC-F38B-4D15-9B50-ABFC67DD1E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3872C156-E37E-459F-B65F-BA60D60C0A39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="58">
   <si>
     <t>NAME_OF_THE_CAMPUS</t>
   </si>
@@ -158,7 +158,55 @@
     <t>TUMKUR</t>
   </si>
   <si>
-    <t>SR_ELITE</t>
+    <t>SR ELITE</t>
+  </si>
+  <si>
+    <t>BANASWADI</t>
+  </si>
+  <si>
+    <t>HEGDENAGAR</t>
+  </si>
+  <si>
+    <t>MAGADI ROAD</t>
+  </si>
+  <si>
+    <t>MARTHAHALLI C-120</t>
+  </si>
+  <si>
+    <t>PEENYA DASARAHALLI</t>
+  </si>
+  <si>
+    <t>UTTARAHALLI</t>
+  </si>
+  <si>
+    <t>YESHWANTHPUR</t>
+  </si>
+  <si>
+    <t>KAGGADASPURA</t>
+  </si>
+  <si>
+    <t>BALLARI BOYS</t>
+  </si>
+  <si>
+    <t>BELAGAVI</t>
+  </si>
+  <si>
+    <t>BHAGATHSINGH NAGAR</t>
+  </si>
+  <si>
+    <t>HUBLI</t>
+  </si>
+  <si>
+    <t>HUBLI 2</t>
+  </si>
+  <si>
+    <t>KOLAR</t>
+  </si>
+  <si>
+    <t>DR BS RAO VIDYASOUDHA MYSORE</t>
+  </si>
+  <si>
+    <t>SR AIIMS</t>
   </si>
 </sst>
 </file>
@@ -535,14 +583,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:R56"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.375" customWidth="1"/>
     <col min="2" max="2" width="8.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -598,7 +646,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -624,7 +672,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -674,7 +722,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -721,7 +769,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -768,7 +816,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -815,7 +863,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -865,7 +913,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -894,7 +942,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -947,7 +995,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -988,7 +1036,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -999,7 +1047,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -1049,7 +1097,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>29</v>
       </c>
@@ -1096,7 +1144,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>30</v>
       </c>
@@ -1146,7 +1194,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>31</v>
       </c>
@@ -1157,7 +1205,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>32</v>
       </c>
@@ -1201,7 +1249,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>33</v>
       </c>
@@ -1251,7 +1299,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -1301,7 +1349,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>35</v>
       </c>
@@ -1336,7 +1384,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>36</v>
       </c>
@@ -1377,7 +1425,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>37</v>
       </c>
@@ -1412,7 +1460,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>38</v>
       </c>
@@ -1459,7 +1507,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>39</v>
       </c>
@@ -1500,7 +1548,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>40</v>
       </c>
@@ -1545,6 +1593,1030 @@
       </c>
       <c r="R24">
         <v>69</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25" t="s">
+        <v>57</v>
+      </c>
+      <c r="C25">
+        <v>2026</v>
+      </c>
+      <c r="D25">
+        <v>34</v>
+      </c>
+      <c r="P25">
+        <v>4</v>
+      </c>
+      <c r="Q25">
+        <v>25</v>
+      </c>
+      <c r="R25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26">
+        <v>2026</v>
+      </c>
+      <c r="D26">
+        <v>59</v>
+      </c>
+      <c r="P26">
+        <v>6</v>
+      </c>
+      <c r="Q26">
+        <v>50</v>
+      </c>
+      <c r="R26">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27">
+        <v>2026</v>
+      </c>
+      <c r="D27">
+        <v>54</v>
+      </c>
+      <c r="K27">
+        <v>1</v>
+      </c>
+      <c r="L27">
+        <v>1</v>
+      </c>
+      <c r="M27">
+        <v>2</v>
+      </c>
+      <c r="N27">
+        <v>6</v>
+      </c>
+      <c r="O27">
+        <v>7</v>
+      </c>
+      <c r="P27">
+        <v>9</v>
+      </c>
+      <c r="Q27">
+        <v>40</v>
+      </c>
+      <c r="R27">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28">
+        <v>2026</v>
+      </c>
+      <c r="D28">
+        <v>46</v>
+      </c>
+      <c r="M28">
+        <v>1</v>
+      </c>
+      <c r="N28">
+        <v>1</v>
+      </c>
+      <c r="O28">
+        <v>3</v>
+      </c>
+      <c r="P28">
+        <v>8</v>
+      </c>
+      <c r="Q28">
+        <v>34</v>
+      </c>
+      <c r="R28">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>20</v>
+      </c>
+      <c r="B29" t="s">
+        <v>57</v>
+      </c>
+      <c r="C29">
+        <v>2026</v>
+      </c>
+      <c r="D29">
+        <v>155</v>
+      </c>
+      <c r="M29">
+        <v>5</v>
+      </c>
+      <c r="N29">
+        <v>10</v>
+      </c>
+      <c r="O29">
+        <v>18</v>
+      </c>
+      <c r="P29">
+        <v>35</v>
+      </c>
+      <c r="Q29">
+        <v>130</v>
+      </c>
+      <c r="R29">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>21</v>
+      </c>
+      <c r="B30" t="s">
+        <v>57</v>
+      </c>
+      <c r="C30">
+        <v>2026</v>
+      </c>
+      <c r="D30">
+        <v>21</v>
+      </c>
+      <c r="L30">
+        <v>1</v>
+      </c>
+      <c r="M30">
+        <v>1</v>
+      </c>
+      <c r="N30">
+        <v>2</v>
+      </c>
+      <c r="O30">
+        <v>2</v>
+      </c>
+      <c r="P30">
+        <v>7</v>
+      </c>
+      <c r="Q30">
+        <v>15</v>
+      </c>
+      <c r="R30">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>43</v>
+      </c>
+      <c r="B31" t="s">
+        <v>57</v>
+      </c>
+      <c r="C31">
+        <v>2026</v>
+      </c>
+      <c r="D31">
+        <v>39</v>
+      </c>
+      <c r="H31">
+        <v>1</v>
+      </c>
+      <c r="I31">
+        <v>1</v>
+      </c>
+      <c r="J31">
+        <v>2</v>
+      </c>
+      <c r="K31">
+        <v>4</v>
+      </c>
+      <c r="L31">
+        <v>4</v>
+      </c>
+      <c r="M31">
+        <v>5</v>
+      </c>
+      <c r="N31">
+        <v>8</v>
+      </c>
+      <c r="O31">
+        <v>9</v>
+      </c>
+      <c r="P31">
+        <v>16</v>
+      </c>
+      <c r="Q31">
+        <v>31</v>
+      </c>
+      <c r="R31">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>22</v>
+      </c>
+      <c r="B32" t="s">
+        <v>57</v>
+      </c>
+      <c r="C32">
+        <v>2026</v>
+      </c>
+      <c r="D32">
+        <v>44</v>
+      </c>
+      <c r="J32">
+        <v>1</v>
+      </c>
+      <c r="K32">
+        <v>2</v>
+      </c>
+      <c r="L32">
+        <v>2</v>
+      </c>
+      <c r="M32">
+        <v>2</v>
+      </c>
+      <c r="N32">
+        <v>4</v>
+      </c>
+      <c r="O32">
+        <v>8</v>
+      </c>
+      <c r="P32">
+        <v>24</v>
+      </c>
+      <c r="Q32">
+        <v>38</v>
+      </c>
+      <c r="R32">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>23</v>
+      </c>
+      <c r="B33" t="s">
+        <v>57</v>
+      </c>
+      <c r="C33">
+        <v>2026</v>
+      </c>
+      <c r="D33">
+        <v>52</v>
+      </c>
+      <c r="N33">
+        <v>2</v>
+      </c>
+      <c r="O33">
+        <v>6</v>
+      </c>
+      <c r="P33">
+        <v>8</v>
+      </c>
+      <c r="Q33">
+        <v>35</v>
+      </c>
+      <c r="R33">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>24</v>
+      </c>
+      <c r="B34" t="s">
+        <v>57</v>
+      </c>
+      <c r="C34">
+        <v>2026</v>
+      </c>
+      <c r="D34">
+        <v>25</v>
+      </c>
+      <c r="N34">
+        <v>1</v>
+      </c>
+      <c r="O34">
+        <v>2</v>
+      </c>
+      <c r="P34">
+        <v>6</v>
+      </c>
+      <c r="Q34">
+        <v>19</v>
+      </c>
+      <c r="R34">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>27</v>
+      </c>
+      <c r="B35" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35">
+        <v>2026</v>
+      </c>
+      <c r="D35">
+        <v>75</v>
+      </c>
+      <c r="K35">
+        <v>1</v>
+      </c>
+      <c r="L35">
+        <v>3</v>
+      </c>
+      <c r="M35">
+        <v>4</v>
+      </c>
+      <c r="N35">
+        <v>11</v>
+      </c>
+      <c r="O35">
+        <v>19</v>
+      </c>
+      <c r="P35">
+        <v>26</v>
+      </c>
+      <c r="Q35">
+        <v>63</v>
+      </c>
+      <c r="R35">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>44</v>
+      </c>
+      <c r="B36" t="s">
+        <v>57</v>
+      </c>
+      <c r="C36">
+        <v>2026</v>
+      </c>
+      <c r="D36">
+        <v>38</v>
+      </c>
+      <c r="M36">
+        <v>1</v>
+      </c>
+      <c r="N36">
+        <v>5</v>
+      </c>
+      <c r="O36">
+        <v>6</v>
+      </c>
+      <c r="P36">
+        <v>14</v>
+      </c>
+      <c r="Q36">
+        <v>35</v>
+      </c>
+      <c r="R36">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>45</v>
+      </c>
+      <c r="B37" t="s">
+        <v>57</v>
+      </c>
+      <c r="C37">
+        <v>2026</v>
+      </c>
+      <c r="D37">
+        <v>66</v>
+      </c>
+      <c r="J37">
+        <v>1</v>
+      </c>
+      <c r="K37">
+        <v>1</v>
+      </c>
+      <c r="L37">
+        <v>3</v>
+      </c>
+      <c r="M37">
+        <v>4</v>
+      </c>
+      <c r="N37">
+        <v>12</v>
+      </c>
+      <c r="O37">
+        <v>17</v>
+      </c>
+      <c r="P37">
+        <v>30</v>
+      </c>
+      <c r="Q37">
+        <v>55</v>
+      </c>
+      <c r="R37">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>29</v>
+      </c>
+      <c r="B38" t="s">
+        <v>57</v>
+      </c>
+      <c r="C38">
+        <v>2026</v>
+      </c>
+      <c r="D38">
+        <v>93</v>
+      </c>
+      <c r="M38">
+        <v>1</v>
+      </c>
+      <c r="N38">
+        <v>4</v>
+      </c>
+      <c r="O38">
+        <v>13</v>
+      </c>
+      <c r="P38">
+        <v>21</v>
+      </c>
+      <c r="Q38">
+        <v>75</v>
+      </c>
+      <c r="R38">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>46</v>
+      </c>
+      <c r="B39" t="s">
+        <v>57</v>
+      </c>
+      <c r="C39">
+        <v>2026</v>
+      </c>
+      <c r="D39">
+        <v>49</v>
+      </c>
+      <c r="J39">
+        <v>1</v>
+      </c>
+      <c r="K39">
+        <v>1</v>
+      </c>
+      <c r="L39">
+        <v>1</v>
+      </c>
+      <c r="M39">
+        <v>2</v>
+      </c>
+      <c r="N39">
+        <v>4</v>
+      </c>
+      <c r="O39">
+        <v>6</v>
+      </c>
+      <c r="P39">
+        <v>13</v>
+      </c>
+      <c r="Q39">
+        <v>43</v>
+      </c>
+      <c r="R39">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>30</v>
+      </c>
+      <c r="B40" t="s">
+        <v>57</v>
+      </c>
+      <c r="C40">
+        <v>2026</v>
+      </c>
+      <c r="D40">
+        <v>119</v>
+      </c>
+      <c r="M40">
+        <v>3</v>
+      </c>
+      <c r="N40">
+        <v>5</v>
+      </c>
+      <c r="O40">
+        <v>10</v>
+      </c>
+      <c r="P40">
+        <v>12</v>
+      </c>
+      <c r="Q40">
+        <v>100</v>
+      </c>
+      <c r="R40">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>47</v>
+      </c>
+      <c r="B41" t="s">
+        <v>57</v>
+      </c>
+      <c r="C41">
+        <v>2026</v>
+      </c>
+      <c r="D41">
+        <v>48</v>
+      </c>
+      <c r="H41">
+        <v>1</v>
+      </c>
+      <c r="I41">
+        <v>2</v>
+      </c>
+      <c r="J41">
+        <v>3</v>
+      </c>
+      <c r="K41">
+        <v>4</v>
+      </c>
+      <c r="L41">
+        <v>4</v>
+      </c>
+      <c r="M41">
+        <v>5</v>
+      </c>
+      <c r="N41">
+        <v>6</v>
+      </c>
+      <c r="O41">
+        <v>11</v>
+      </c>
+      <c r="P41">
+        <v>20</v>
+      </c>
+      <c r="Q41">
+        <v>46</v>
+      </c>
+      <c r="R41">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>33</v>
+      </c>
+      <c r="B42" t="s">
+        <v>57</v>
+      </c>
+      <c r="C42">
+        <v>2026</v>
+      </c>
+      <c r="D42">
+        <v>63</v>
+      </c>
+      <c r="L42">
+        <v>1</v>
+      </c>
+      <c r="M42">
+        <v>2</v>
+      </c>
+      <c r="N42">
+        <v>4</v>
+      </c>
+      <c r="O42">
+        <v>9</v>
+      </c>
+      <c r="P42">
+        <v>16</v>
+      </c>
+      <c r="Q42">
+        <v>54</v>
+      </c>
+      <c r="R42">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>48</v>
+      </c>
+      <c r="B43" t="s">
+        <v>57</v>
+      </c>
+      <c r="C43">
+        <v>2026</v>
+      </c>
+      <c r="D43">
+        <v>31</v>
+      </c>
+      <c r="O43">
+        <v>1</v>
+      </c>
+      <c r="P43">
+        <v>4</v>
+      </c>
+      <c r="Q43">
+        <v>23</v>
+      </c>
+      <c r="R43">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>34</v>
+      </c>
+      <c r="B44" t="s">
+        <v>57</v>
+      </c>
+      <c r="C44">
+        <v>2026</v>
+      </c>
+      <c r="D44">
+        <v>101</v>
+      </c>
+      <c r="L44">
+        <v>1</v>
+      </c>
+      <c r="M44">
+        <v>1</v>
+      </c>
+      <c r="N44">
+        <v>2</v>
+      </c>
+      <c r="O44">
+        <v>10</v>
+      </c>
+      <c r="P44">
+        <v>15</v>
+      </c>
+      <c r="Q44">
+        <v>75</v>
+      </c>
+      <c r="R44">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>49</v>
+      </c>
+      <c r="B45" t="s">
+        <v>57</v>
+      </c>
+      <c r="C45">
+        <v>2026</v>
+      </c>
+      <c r="D45">
+        <v>39</v>
+      </c>
+      <c r="H45">
+        <v>1</v>
+      </c>
+      <c r="I45">
+        <v>1</v>
+      </c>
+      <c r="J45">
+        <v>3</v>
+      </c>
+      <c r="K45">
+        <v>3</v>
+      </c>
+      <c r="L45">
+        <v>4</v>
+      </c>
+      <c r="M45">
+        <v>5</v>
+      </c>
+      <c r="N45">
+        <v>11</v>
+      </c>
+      <c r="O45">
+        <v>15</v>
+      </c>
+      <c r="P45">
+        <v>23</v>
+      </c>
+      <c r="Q45">
+        <v>35</v>
+      </c>
+      <c r="R45">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>52</v>
+      </c>
+      <c r="B46" t="s">
+        <v>57</v>
+      </c>
+      <c r="C46">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>35</v>
+      </c>
+      <c r="B47" t="s">
+        <v>57</v>
+      </c>
+      <c r="C47">
+        <v>2026</v>
+      </c>
+      <c r="D47">
+        <v>47</v>
+      </c>
+      <c r="N47">
+        <v>1</v>
+      </c>
+      <c r="O47">
+        <v>4</v>
+      </c>
+      <c r="P47">
+        <v>10</v>
+      </c>
+      <c r="Q47">
+        <v>35</v>
+      </c>
+      <c r="R47">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>36</v>
+      </c>
+      <c r="B48" t="s">
+        <v>57</v>
+      </c>
+      <c r="C48">
+        <v>2026</v>
+      </c>
+      <c r="D48">
+        <v>46</v>
+      </c>
+      <c r="O48">
+        <v>1</v>
+      </c>
+      <c r="P48">
+        <v>9</v>
+      </c>
+      <c r="Q48">
+        <v>32</v>
+      </c>
+      <c r="R48">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>53</v>
+      </c>
+      <c r="B49" t="s">
+        <v>57</v>
+      </c>
+      <c r="C49">
+        <v>2026</v>
+      </c>
+      <c r="D49">
+        <v>41</v>
+      </c>
+      <c r="J49">
+        <v>1</v>
+      </c>
+      <c r="K49">
+        <v>2</v>
+      </c>
+      <c r="L49">
+        <v>2</v>
+      </c>
+      <c r="M49">
+        <v>2</v>
+      </c>
+      <c r="N49">
+        <v>5</v>
+      </c>
+      <c r="O49">
+        <v>9</v>
+      </c>
+      <c r="P49">
+        <v>14</v>
+      </c>
+      <c r="Q49">
+        <v>35</v>
+      </c>
+      <c r="R49">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>54</v>
+      </c>
+      <c r="B50" t="s">
+        <v>57</v>
+      </c>
+      <c r="C50">
+        <v>2026</v>
+      </c>
+      <c r="D50">
+        <v>52</v>
+      </c>
+      <c r="O50">
+        <v>1</v>
+      </c>
+      <c r="P50">
+        <v>5</v>
+      </c>
+      <c r="Q50">
+        <v>34</v>
+      </c>
+      <c r="R50">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>55</v>
+      </c>
+      <c r="B51" t="s">
+        <v>57</v>
+      </c>
+      <c r="C51">
+        <v>2026</v>
+      </c>
+      <c r="D51">
+        <v>42</v>
+      </c>
+      <c r="O51">
+        <v>3</v>
+      </c>
+      <c r="P51">
+        <v>8</v>
+      </c>
+      <c r="Q51">
+        <v>38</v>
+      </c>
+      <c r="R51">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>37</v>
+      </c>
+      <c r="B52" t="s">
+        <v>57</v>
+      </c>
+      <c r="C52">
+        <v>2026</v>
+      </c>
+      <c r="D52">
+        <v>42</v>
+      </c>
+      <c r="O52">
+        <v>1</v>
+      </c>
+      <c r="P52">
+        <v>6</v>
+      </c>
+      <c r="Q52">
+        <v>31</v>
+      </c>
+      <c r="R52">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>38</v>
+      </c>
+      <c r="B53" t="s">
+        <v>57</v>
+      </c>
+      <c r="C53">
+        <v>2026</v>
+      </c>
+      <c r="D53">
+        <v>59</v>
+      </c>
+      <c r="N53">
+        <v>2</v>
+      </c>
+      <c r="O53">
+        <v>6</v>
+      </c>
+      <c r="P53">
+        <v>13</v>
+      </c>
+      <c r="Q53">
+        <v>45</v>
+      </c>
+      <c r="R53">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>39</v>
+      </c>
+      <c r="B54" t="s">
+        <v>57</v>
+      </c>
+      <c r="C54">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>56</v>
+      </c>
+      <c r="B55" t="s">
+        <v>57</v>
+      </c>
+      <c r="C55">
+        <v>2026</v>
+      </c>
+      <c r="D55">
+        <v>35</v>
+      </c>
+      <c r="N55">
+        <v>3</v>
+      </c>
+      <c r="O55">
+        <v>5</v>
+      </c>
+      <c r="P55">
+        <v>18</v>
+      </c>
+      <c r="Q55">
+        <v>34</v>
+      </c>
+      <c r="R55">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>40</v>
+      </c>
+      <c r="B56" t="s">
+        <v>57</v>
+      </c>
+      <c r="C56">
+        <v>2026</v>
+      </c>
+      <c r="D56">
+        <v>121</v>
+      </c>
+      <c r="L56">
+        <v>1</v>
+      </c>
+      <c r="M56">
+        <v>2</v>
+      </c>
+      <c r="N56">
+        <v>5</v>
+      </c>
+      <c r="O56">
+        <v>10</v>
+      </c>
+      <c r="P56">
+        <v>13</v>
+      </c>
+      <c r="Q56">
+        <v>100</v>
+      </c>
+      <c r="R56">
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-deploy updates: Wed 10/07/2026 13:44:18.58
</commit_message>
<xml_diff>
--- a/NEET_2026_Targets_Template.xlsx
+++ b/NEET_2026_Targets_Template.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\NEET Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3872C156-E37E-459F-B65F-BA60D60C0A39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7568E897-531C-4DCF-ADBF-DA2A5376E1AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Targets" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Targets!$A$1:$AA$80</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -33,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="64">
   <si>
     <t>NAME_OF_THE_CAMPUS</t>
   </si>
@@ -207,6 +210,24 @@
   </si>
   <si>
     <t>SR AIIMS</t>
+  </si>
+  <si>
+    <t>LTC</t>
+  </si>
+  <si>
+    <t>&gt;= 480M</t>
+  </si>
+  <si>
+    <t>&gt;= 370M</t>
+  </si>
+  <si>
+    <t>&gt;= 350M</t>
+  </si>
+  <si>
+    <t>HEBBAL</t>
+  </si>
+  <si>
+    <t>JR ELITE</t>
   </si>
 </sst>
 </file>
@@ -583,14 +604,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R56"/>
+  <dimension ref="A1:U80"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.375" customWidth="1"/>
     <col min="2" max="2" width="8.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -634,19 +655,28 @@
         <v>13</v>
       </c>
       <c r="O1" t="s">
+        <v>59</v>
+      </c>
+      <c r="P1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
+        <v>60</v>
+      </c>
+      <c r="S1" t="s">
+        <v>61</v>
+      </c>
+      <c r="T1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="U1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -659,20 +689,20 @@
       <c r="D2">
         <v>30</v>
       </c>
-      <c r="O2">
-        <v>1</v>
-      </c>
       <c r="P2">
+        <v>1</v>
+      </c>
+      <c r="Q2">
         <v>5</v>
       </c>
-      <c r="Q2">
+      <c r="T2">
         <v>30</v>
       </c>
-      <c r="R2">
+      <c r="U2">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -709,20 +739,20 @@
       <c r="N3">
         <v>45</v>
       </c>
-      <c r="O3">
+      <c r="P3">
         <v>56</v>
       </c>
-      <c r="P3">
+      <c r="Q3">
         <v>61</v>
       </c>
-      <c r="Q3">
+      <c r="T3">
         <v>73</v>
       </c>
-      <c r="R3">
+      <c r="U3">
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -756,20 +786,20 @@
       <c r="N4">
         <v>36</v>
       </c>
-      <c r="O4">
+      <c r="P4">
         <v>50</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>150</v>
       </c>
-      <c r="Q4">
+      <c r="T4">
         <v>216</v>
       </c>
-      <c r="R4">
+      <c r="U4">
         <v>216</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -803,20 +833,20 @@
       <c r="N5">
         <v>20</v>
       </c>
-      <c r="O5">
+      <c r="P5">
         <v>26</v>
       </c>
-      <c r="P5">
+      <c r="Q5">
         <v>45</v>
       </c>
-      <c r="Q5">
+      <c r="T5">
         <v>64</v>
       </c>
-      <c r="R5">
+      <c r="U5">
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -850,20 +880,20 @@
       <c r="N6">
         <v>17</v>
       </c>
-      <c r="O6">
+      <c r="P6">
         <v>19</v>
       </c>
-      <c r="P6">
+      <c r="Q6">
         <v>38</v>
       </c>
-      <c r="Q6">
+      <c r="T6">
         <v>54</v>
       </c>
-      <c r="R6">
+      <c r="U6">
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -900,20 +930,20 @@
       <c r="N7">
         <v>36</v>
       </c>
-      <c r="O7">
+      <c r="P7">
         <v>43</v>
       </c>
-      <c r="P7">
+      <c r="Q7">
         <v>65</v>
       </c>
-      <c r="Q7">
+      <c r="T7">
         <v>101</v>
       </c>
-      <c r="R7">
+      <c r="U7">
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -929,20 +959,20 @@
       <c r="N8">
         <v>4</v>
       </c>
-      <c r="O8">
+      <c r="P8">
         <v>4</v>
       </c>
-      <c r="P8">
+      <c r="Q8">
         <v>15</v>
       </c>
-      <c r="Q8">
+      <c r="T8">
         <v>24</v>
       </c>
-      <c r="R8">
+      <c r="U8">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -982,20 +1012,20 @@
       <c r="N9">
         <v>15</v>
       </c>
-      <c r="O9">
+      <c r="P9">
         <v>24</v>
       </c>
-      <c r="P9">
+      <c r="Q9">
         <v>52</v>
       </c>
-      <c r="Q9">
+      <c r="T9">
         <v>98</v>
       </c>
-      <c r="R9">
+      <c r="U9">
         <v>98</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -1023,20 +1053,20 @@
       <c r="N10">
         <v>2</v>
       </c>
-      <c r="O10">
+      <c r="P10">
         <v>4</v>
       </c>
-      <c r="P10">
+      <c r="Q10">
         <v>20</v>
       </c>
-      <c r="Q10">
+      <c r="T10">
         <v>46</v>
       </c>
-      <c r="R10">
+      <c r="U10">
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -1047,7 +1077,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -1084,20 +1114,20 @@
       <c r="N12">
         <v>89</v>
       </c>
-      <c r="O12">
+      <c r="P12">
         <v>109</v>
       </c>
-      <c r="P12">
+      <c r="Q12">
         <v>135</v>
       </c>
-      <c r="Q12">
+      <c r="T12">
         <v>164</v>
       </c>
-      <c r="R12">
+      <c r="U12">
         <v>164</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>29</v>
       </c>
@@ -1131,20 +1161,20 @@
       <c r="N13">
         <v>24</v>
       </c>
-      <c r="O13">
+      <c r="P13">
         <v>32</v>
       </c>
-      <c r="P13">
+      <c r="Q13">
         <v>44</v>
       </c>
-      <c r="Q13">
+      <c r="T13">
         <v>60</v>
       </c>
-      <c r="R13">
+      <c r="U13">
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>30</v>
       </c>
@@ -1181,20 +1211,20 @@
       <c r="N14">
         <v>23</v>
       </c>
-      <c r="O14">
+      <c r="P14">
         <v>30</v>
       </c>
-      <c r="P14">
+      <c r="Q14">
         <v>45</v>
       </c>
-      <c r="Q14">
+      <c r="T14">
         <v>53</v>
       </c>
-      <c r="R14">
+      <c r="U14">
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>31</v>
       </c>
@@ -1205,7 +1235,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>32</v>
       </c>
@@ -1236,20 +1266,20 @@
       <c r="N16">
         <v>3</v>
       </c>
-      <c r="O16">
+      <c r="P16">
         <v>5</v>
       </c>
-      <c r="P16">
+      <c r="Q16">
         <v>25</v>
       </c>
-      <c r="Q16">
+      <c r="T16">
         <v>50</v>
       </c>
-      <c r="R16">
+      <c r="U16">
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>33</v>
       </c>
@@ -1286,20 +1316,20 @@
       <c r="N17">
         <v>17</v>
       </c>
-      <c r="O17">
+      <c r="P17">
         <v>21</v>
       </c>
-      <c r="P17">
+      <c r="Q17">
         <v>31</v>
       </c>
-      <c r="Q17">
+      <c r="T17">
         <v>44</v>
       </c>
-      <c r="R17">
+      <c r="U17">
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -1336,20 +1366,20 @@
       <c r="N18">
         <v>32</v>
       </c>
-      <c r="O18">
+      <c r="P18">
         <v>50</v>
       </c>
-      <c r="P18">
+      <c r="Q18">
         <v>100</v>
       </c>
-      <c r="Q18">
+      <c r="T18">
         <v>191</v>
       </c>
-      <c r="R18">
+      <c r="U18">
         <v>191</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>35</v>
       </c>
@@ -1371,20 +1401,20 @@
       <c r="N19">
         <v>1</v>
       </c>
-      <c r="O19">
-        <v>1</v>
-      </c>
       <c r="P19">
+        <v>1</v>
+      </c>
+      <c r="Q19">
         <v>5</v>
       </c>
-      <c r="Q19">
+      <c r="T19">
         <v>7</v>
       </c>
-      <c r="R19">
+      <c r="U19">
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>36</v>
       </c>
@@ -1412,20 +1442,20 @@
       <c r="N20">
         <v>5</v>
       </c>
-      <c r="O20">
+      <c r="P20">
         <v>13</v>
       </c>
-      <c r="P20">
+      <c r="Q20">
         <v>25</v>
       </c>
-      <c r="Q20">
+      <c r="T20">
         <v>33</v>
       </c>
-      <c r="R20">
+      <c r="U20">
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>37</v>
       </c>
@@ -1447,20 +1477,20 @@
       <c r="N21">
         <v>2</v>
       </c>
-      <c r="O21">
+      <c r="P21">
         <v>4</v>
       </c>
-      <c r="P21">
+      <c r="Q21">
         <v>20</v>
       </c>
-      <c r="Q21">
+      <c r="T21">
         <v>34</v>
       </c>
-      <c r="R21">
+      <c r="U21">
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>38</v>
       </c>
@@ -1494,20 +1524,20 @@
       <c r="N22">
         <v>7</v>
       </c>
-      <c r="O22">
+      <c r="P22">
         <v>11</v>
       </c>
-      <c r="P22">
+      <c r="Q22">
         <v>21</v>
       </c>
-      <c r="Q22">
+      <c r="T22">
         <v>42</v>
       </c>
-      <c r="R22">
+      <c r="U22">
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>39</v>
       </c>
@@ -1535,20 +1565,20 @@
       <c r="N23">
         <v>4</v>
       </c>
-      <c r="O23">
+      <c r="P23">
         <v>7</v>
       </c>
-      <c r="P23">
+      <c r="Q23">
         <v>26</v>
       </c>
-      <c r="Q23">
+      <c r="T23">
         <v>54</v>
       </c>
-      <c r="R23">
+      <c r="U23">
         <v>54</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>40</v>
       </c>
@@ -1582,20 +1612,20 @@
       <c r="N24">
         <v>13</v>
       </c>
-      <c r="O24">
+      <c r="P24">
         <v>20</v>
       </c>
-      <c r="P24">
+      <c r="Q24">
         <v>40</v>
       </c>
-      <c r="Q24">
+      <c r="T24">
         <v>69</v>
       </c>
-      <c r="R24">
+      <c r="U24">
         <v>69</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>50</v>
       </c>
@@ -1608,17 +1638,17 @@
       <c r="D25">
         <v>34</v>
       </c>
-      <c r="P25">
+      <c r="Q25">
         <v>4</v>
       </c>
-      <c r="Q25">
+      <c r="T25">
         <v>25</v>
       </c>
-      <c r="R25">
+      <c r="U25">
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>18</v>
       </c>
@@ -1631,17 +1661,17 @@
       <c r="D26">
         <v>59</v>
       </c>
-      <c r="P26">
+      <c r="Q26">
         <v>6</v>
       </c>
-      <c r="Q26">
+      <c r="T26">
         <v>50</v>
       </c>
-      <c r="R26">
+      <c r="U26">
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>51</v>
       </c>
@@ -1666,20 +1696,20 @@
       <c r="N27">
         <v>6</v>
       </c>
-      <c r="O27">
+      <c r="P27">
         <v>7</v>
       </c>
-      <c r="P27">
+      <c r="Q27">
         <v>9</v>
       </c>
-      <c r="Q27">
+      <c r="T27">
         <v>40</v>
       </c>
-      <c r="R27">
+      <c r="U27">
         <v>54</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>42</v>
       </c>
@@ -1698,20 +1728,20 @@
       <c r="N28">
         <v>1</v>
       </c>
-      <c r="O28">
+      <c r="P28">
         <v>3</v>
       </c>
-      <c r="P28">
+      <c r="Q28">
         <v>8</v>
       </c>
-      <c r="Q28">
+      <c r="T28">
         <v>34</v>
       </c>
-      <c r="R28">
+      <c r="U28">
         <v>46</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>20</v>
       </c>
@@ -1730,20 +1760,20 @@
       <c r="N29">
         <v>10</v>
       </c>
-      <c r="O29">
+      <c r="P29">
         <v>18</v>
       </c>
-      <c r="P29">
+      <c r="Q29">
         <v>35</v>
       </c>
-      <c r="Q29">
+      <c r="T29">
         <v>130</v>
       </c>
-      <c r="R29">
+      <c r="U29">
         <v>155</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>21</v>
       </c>
@@ -1765,20 +1795,20 @@
       <c r="N30">
         <v>2</v>
       </c>
-      <c r="O30">
-        <v>2</v>
-      </c>
       <c r="P30">
+        <v>2</v>
+      </c>
+      <c r="Q30">
         <v>7</v>
       </c>
-      <c r="Q30">
+      <c r="T30">
         <v>15</v>
       </c>
-      <c r="R30">
+      <c r="U30">
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>43</v>
       </c>
@@ -1812,20 +1842,20 @@
       <c r="N31">
         <v>8</v>
       </c>
-      <c r="O31">
+      <c r="P31">
         <v>9</v>
       </c>
-      <c r="P31">
+      <c r="Q31">
         <v>16</v>
       </c>
-      <c r="Q31">
+      <c r="T31">
         <v>31</v>
       </c>
-      <c r="R31">
+      <c r="U31">
         <v>39</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -1853,20 +1883,20 @@
       <c r="N32">
         <v>4</v>
       </c>
-      <c r="O32">
+      <c r="P32">
         <v>8</v>
       </c>
-      <c r="P32">
+      <c r="Q32">
         <v>24</v>
       </c>
-      <c r="Q32">
+      <c r="T32">
         <v>38</v>
       </c>
-      <c r="R32">
+      <c r="U32">
         <v>44</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -1882,20 +1912,20 @@
       <c r="N33">
         <v>2</v>
       </c>
-      <c r="O33">
+      <c r="P33">
         <v>6</v>
       </c>
-      <c r="P33">
+      <c r="Q33">
         <v>8</v>
       </c>
-      <c r="Q33">
+      <c r="T33">
         <v>35</v>
       </c>
-      <c r="R33">
+      <c r="U33">
         <v>52</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>24</v>
       </c>
@@ -1911,20 +1941,20 @@
       <c r="N34">
         <v>1</v>
       </c>
-      <c r="O34">
-        <v>2</v>
-      </c>
       <c r="P34">
+        <v>2</v>
+      </c>
+      <c r="Q34">
         <v>6</v>
       </c>
-      <c r="Q34">
+      <c r="T34">
         <v>19</v>
       </c>
-      <c r="R34">
+      <c r="U34">
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>27</v>
       </c>
@@ -1949,20 +1979,20 @@
       <c r="N35">
         <v>11</v>
       </c>
-      <c r="O35">
+      <c r="P35">
         <v>19</v>
       </c>
-      <c r="P35">
+      <c r="Q35">
         <v>26</v>
       </c>
-      <c r="Q35">
+      <c r="T35">
         <v>63</v>
       </c>
-      <c r="R35">
+      <c r="U35">
         <v>75</v>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>44</v>
       </c>
@@ -1981,20 +2011,20 @@
       <c r="N36">
         <v>5</v>
       </c>
-      <c r="O36">
+      <c r="P36">
         <v>6</v>
       </c>
-      <c r="P36">
+      <c r="Q36">
         <v>14</v>
       </c>
-      <c r="Q36">
+      <c r="T36">
         <v>35</v>
       </c>
-      <c r="R36">
+      <c r="U36">
         <v>38</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>45</v>
       </c>
@@ -2022,20 +2052,20 @@
       <c r="N37">
         <v>12</v>
       </c>
-      <c r="O37">
+      <c r="P37">
         <v>17</v>
       </c>
-      <c r="P37">
+      <c r="Q37">
         <v>30</v>
       </c>
-      <c r="Q37">
+      <c r="T37">
         <v>55</v>
       </c>
-      <c r="R37">
+      <c r="U37">
         <v>66</v>
       </c>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>29</v>
       </c>
@@ -2054,20 +2084,20 @@
       <c r="N38">
         <v>4</v>
       </c>
-      <c r="O38">
+      <c r="P38">
         <v>13</v>
       </c>
-      <c r="P38">
+      <c r="Q38">
         <v>21</v>
       </c>
-      <c r="Q38">
+      <c r="T38">
         <v>75</v>
       </c>
-      <c r="R38">
+      <c r="U38">
         <v>93</v>
       </c>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>46</v>
       </c>
@@ -2095,20 +2125,20 @@
       <c r="N39">
         <v>4</v>
       </c>
-      <c r="O39">
+      <c r="P39">
         <v>6</v>
       </c>
-      <c r="P39">
+      <c r="Q39">
         <v>13</v>
       </c>
-      <c r="Q39">
+      <c r="T39">
         <v>43</v>
       </c>
-      <c r="R39">
+      <c r="U39">
         <v>49</v>
       </c>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>30</v>
       </c>
@@ -2127,20 +2157,20 @@
       <c r="N40">
         <v>5</v>
       </c>
-      <c r="O40">
+      <c r="P40">
         <v>10</v>
       </c>
-      <c r="P40">
+      <c r="Q40">
         <v>12</v>
       </c>
-      <c r="Q40">
+      <c r="T40">
         <v>100</v>
       </c>
-      <c r="R40">
+      <c r="U40">
         <v>119</v>
       </c>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>47</v>
       </c>
@@ -2174,20 +2204,20 @@
       <c r="N41">
         <v>6</v>
       </c>
-      <c r="O41">
+      <c r="P41">
         <v>11</v>
       </c>
-      <c r="P41">
+      <c r="Q41">
         <v>20</v>
       </c>
-      <c r="Q41">
+      <c r="T41">
         <v>46</v>
       </c>
-      <c r="R41">
+      <c r="U41">
         <v>48</v>
       </c>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>33</v>
       </c>
@@ -2209,20 +2239,20 @@
       <c r="N42">
         <v>4</v>
       </c>
-      <c r="O42">
+      <c r="P42">
         <v>9</v>
       </c>
-      <c r="P42">
+      <c r="Q42">
         <v>16</v>
       </c>
-      <c r="Q42">
+      <c r="T42">
         <v>54</v>
       </c>
-      <c r="R42">
+      <c r="U42">
         <v>63</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>48</v>
       </c>
@@ -2235,20 +2265,20 @@
       <c r="D43">
         <v>31</v>
       </c>
-      <c r="O43">
-        <v>1</v>
-      </c>
       <c r="P43">
+        <v>1</v>
+      </c>
+      <c r="Q43">
         <v>4</v>
       </c>
-      <c r="Q43">
+      <c r="T43">
         <v>23</v>
       </c>
-      <c r="R43">
+      <c r="U43">
         <v>31</v>
       </c>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>34</v>
       </c>
@@ -2270,20 +2300,20 @@
       <c r="N44">
         <v>2</v>
       </c>
-      <c r="O44">
+      <c r="P44">
         <v>10</v>
       </c>
-      <c r="P44">
+      <c r="Q44">
         <v>15</v>
       </c>
-      <c r="Q44">
+      <c r="T44">
         <v>75</v>
       </c>
-      <c r="R44">
+      <c r="U44">
         <v>101</v>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>49</v>
       </c>
@@ -2317,20 +2347,20 @@
       <c r="N45">
         <v>11</v>
       </c>
-      <c r="O45">
+      <c r="P45">
         <v>15</v>
       </c>
-      <c r="P45">
+      <c r="Q45">
         <v>23</v>
       </c>
-      <c r="Q45">
+      <c r="T45">
         <v>35</v>
       </c>
-      <c r="R45">
+      <c r="U45">
         <v>39</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>52</v>
       </c>
@@ -2341,7 +2371,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>35</v>
       </c>
@@ -2357,20 +2387,20 @@
       <c r="N47">
         <v>1</v>
       </c>
-      <c r="O47">
+      <c r="P47">
         <v>4</v>
       </c>
-      <c r="P47">
+      <c r="Q47">
         <v>10</v>
       </c>
-      <c r="Q47">
+      <c r="T47">
         <v>35</v>
       </c>
-      <c r="R47">
+      <c r="U47">
         <v>47</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>36</v>
       </c>
@@ -2383,20 +2413,20 @@
       <c r="D48">
         <v>46</v>
       </c>
-      <c r="O48">
-        <v>1</v>
-      </c>
       <c r="P48">
+        <v>1</v>
+      </c>
+      <c r="Q48">
         <v>9</v>
       </c>
-      <c r="Q48">
+      <c r="T48">
         <v>32</v>
       </c>
-      <c r="R48">
+      <c r="U48">
         <v>46</v>
       </c>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>53</v>
       </c>
@@ -2424,20 +2454,20 @@
       <c r="N49">
         <v>5</v>
       </c>
-      <c r="O49">
+      <c r="P49">
         <v>9</v>
       </c>
-      <c r="P49">
+      <c r="Q49">
         <v>14</v>
       </c>
-      <c r="Q49">
+      <c r="T49">
         <v>35</v>
       </c>
-      <c r="R49">
+      <c r="U49">
         <v>41</v>
       </c>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>54</v>
       </c>
@@ -2450,20 +2480,20 @@
       <c r="D50">
         <v>52</v>
       </c>
-      <c r="O50">
-        <v>1</v>
-      </c>
       <c r="P50">
+        <v>1</v>
+      </c>
+      <c r="Q50">
         <v>5</v>
       </c>
-      <c r="Q50">
+      <c r="T50">
         <v>34</v>
       </c>
-      <c r="R50">
+      <c r="U50">
         <v>52</v>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>55</v>
       </c>
@@ -2476,20 +2506,20 @@
       <c r="D51">
         <v>42</v>
       </c>
-      <c r="O51">
+      <c r="P51">
         <v>3</v>
       </c>
-      <c r="P51">
+      <c r="Q51">
         <v>8</v>
       </c>
-      <c r="Q51">
+      <c r="T51">
         <v>38</v>
       </c>
-      <c r="R51">
+      <c r="U51">
         <v>42</v>
       </c>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>37</v>
       </c>
@@ -2502,20 +2532,20 @@
       <c r="D52">
         <v>42</v>
       </c>
-      <c r="O52">
-        <v>1</v>
-      </c>
       <c r="P52">
+        <v>1</v>
+      </c>
+      <c r="Q52">
         <v>6</v>
       </c>
-      <c r="Q52">
+      <c r="T52">
         <v>31</v>
       </c>
-      <c r="R52">
+      <c r="U52">
         <v>42</v>
       </c>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>38</v>
       </c>
@@ -2531,20 +2561,20 @@
       <c r="N53">
         <v>2</v>
       </c>
-      <c r="O53">
+      <c r="P53">
         <v>6</v>
       </c>
-      <c r="P53">
+      <c r="Q53">
         <v>13</v>
       </c>
-      <c r="Q53">
+      <c r="T53">
         <v>45</v>
       </c>
-      <c r="R53">
+      <c r="U53">
         <v>59</v>
       </c>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>39</v>
       </c>
@@ -2555,7 +2585,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>56</v>
       </c>
@@ -2571,20 +2601,20 @@
       <c r="N55">
         <v>3</v>
       </c>
-      <c r="O55">
+      <c r="P55">
         <v>5</v>
       </c>
-      <c r="P55">
+      <c r="Q55">
         <v>18</v>
       </c>
-      <c r="Q55">
+      <c r="T55">
         <v>34</v>
       </c>
-      <c r="R55">
+      <c r="U55">
         <v>35</v>
       </c>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>40</v>
       </c>
@@ -2606,23 +2636,1302 @@
       <c r="N56">
         <v>5</v>
       </c>
-      <c r="O56">
+      <c r="P56">
         <v>10</v>
       </c>
-      <c r="P56">
+      <c r="Q56">
         <v>13</v>
       </c>
-      <c r="Q56">
+      <c r="T56">
         <v>100</v>
       </c>
-      <c r="R56">
+      <c r="U56">
         <v>121</v>
       </c>
     </row>
+    <row r="57" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>18</v>
+      </c>
+      <c r="B57" t="s">
+        <v>58</v>
+      </c>
+      <c r="C57">
+        <v>2026</v>
+      </c>
+      <c r="D57">
+        <v>16</v>
+      </c>
+      <c r="K57">
+        <v>1</v>
+      </c>
+      <c r="L57">
+        <v>1</v>
+      </c>
+      <c r="M57">
+        <v>3</v>
+      </c>
+      <c r="N57">
+        <v>5</v>
+      </c>
+      <c r="O57">
+        <v>7</v>
+      </c>
+      <c r="P57">
+        <v>11</v>
+      </c>
+      <c r="Q57">
+        <v>13</v>
+      </c>
+      <c r="R57">
+        <v>13</v>
+      </c>
+      <c r="S57">
+        <v>16</v>
+      </c>
+      <c r="T57">
+        <v>16</v>
+      </c>
+      <c r="U57">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="58" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>51</v>
+      </c>
+      <c r="B58" t="s">
+        <v>58</v>
+      </c>
+      <c r="C58">
+        <v>2026</v>
+      </c>
+      <c r="D58">
+        <v>5</v>
+      </c>
+      <c r="S58">
+        <v>5</v>
+      </c>
+      <c r="T58">
+        <v>5</v>
+      </c>
+      <c r="U58">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>20</v>
+      </c>
+      <c r="B59" t="s">
+        <v>58</v>
+      </c>
+      <c r="C59">
+        <v>2026</v>
+      </c>
+      <c r="D59">
+        <v>52</v>
+      </c>
+      <c r="G59">
+        <v>1</v>
+      </c>
+      <c r="H59">
+        <v>1</v>
+      </c>
+      <c r="I59">
+        <v>8</v>
+      </c>
+      <c r="J59">
+        <v>1</v>
+      </c>
+      <c r="K59">
+        <v>12</v>
+      </c>
+      <c r="L59">
+        <v>15</v>
+      </c>
+      <c r="M59">
+        <v>21</v>
+      </c>
+      <c r="N59">
+        <v>27</v>
+      </c>
+      <c r="O59">
+        <v>28</v>
+      </c>
+      <c r="P59">
+        <v>38</v>
+      </c>
+      <c r="Q59">
+        <v>39</v>
+      </c>
+      <c r="R59">
+        <v>40</v>
+      </c>
+      <c r="S59">
+        <v>52</v>
+      </c>
+      <c r="T59">
+        <v>52</v>
+      </c>
+      <c r="U59">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="60" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>34</v>
+      </c>
+      <c r="B60" t="s">
+        <v>58</v>
+      </c>
+      <c r="C60">
+        <v>2026</v>
+      </c>
+      <c r="D60">
+        <v>32</v>
+      </c>
+      <c r="H60">
+        <v>1</v>
+      </c>
+      <c r="I60">
+        <v>7</v>
+      </c>
+      <c r="J60">
+        <v>2</v>
+      </c>
+      <c r="K60">
+        <v>9</v>
+      </c>
+      <c r="L60">
+        <v>11</v>
+      </c>
+      <c r="M60">
+        <v>13</v>
+      </c>
+      <c r="N60">
+        <v>19</v>
+      </c>
+      <c r="O60">
+        <v>20</v>
+      </c>
+      <c r="P60">
+        <v>27</v>
+      </c>
+      <c r="Q60">
+        <v>28</v>
+      </c>
+      <c r="R60">
+        <v>30</v>
+      </c>
+      <c r="S60">
+        <v>32</v>
+      </c>
+      <c r="T60">
+        <v>32</v>
+      </c>
+      <c r="U60">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="61" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>35</v>
+      </c>
+      <c r="B61" t="s">
+        <v>58</v>
+      </c>
+      <c r="C61">
+        <v>2026</v>
+      </c>
+      <c r="D61">
+        <v>11</v>
+      </c>
+      <c r="N61">
+        <v>1</v>
+      </c>
+      <c r="O61">
+        <v>1</v>
+      </c>
+      <c r="P61">
+        <v>3</v>
+      </c>
+      <c r="Q61">
+        <v>4</v>
+      </c>
+      <c r="R61">
+        <v>5</v>
+      </c>
+      <c r="S61">
+        <v>11</v>
+      </c>
+      <c r="T61">
+        <v>11</v>
+      </c>
+      <c r="U61">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="62" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>36</v>
+      </c>
+      <c r="B62" t="s">
+        <v>58</v>
+      </c>
+      <c r="C62">
+        <v>2026</v>
+      </c>
+      <c r="D62">
+        <v>7</v>
+      </c>
+      <c r="K62">
+        <v>1</v>
+      </c>
+      <c r="L62">
+        <v>1</v>
+      </c>
+      <c r="M62">
+        <v>1</v>
+      </c>
+      <c r="N62">
+        <v>2</v>
+      </c>
+      <c r="O62">
+        <v>3</v>
+      </c>
+      <c r="P62">
+        <v>3</v>
+      </c>
+      <c r="Q62">
+        <v>3</v>
+      </c>
+      <c r="R62">
+        <v>3</v>
+      </c>
+      <c r="S62">
+        <v>7</v>
+      </c>
+      <c r="T62">
+        <v>7</v>
+      </c>
+      <c r="U62">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>19</v>
+      </c>
+      <c r="B63" t="s">
+        <v>63</v>
+      </c>
+      <c r="C63">
+        <v>2026</v>
+      </c>
+      <c r="D63">
+        <v>117</v>
+      </c>
+      <c r="E63">
+        <v>2</v>
+      </c>
+      <c r="F63">
+        <v>5</v>
+      </c>
+      <c r="G63">
+        <v>13</v>
+      </c>
+      <c r="H63">
+        <v>22</v>
+      </c>
+      <c r="I63">
+        <v>22</v>
+      </c>
+      <c r="J63">
+        <v>40</v>
+      </c>
+      <c r="K63">
+        <v>117</v>
+      </c>
+      <c r="L63">
+        <v>52</v>
+      </c>
+      <c r="M63">
+        <v>56</v>
+      </c>
+      <c r="N63">
+        <v>62</v>
+      </c>
+      <c r="P63">
+        <v>64</v>
+      </c>
+      <c r="Q63">
+        <v>67</v>
+      </c>
+      <c r="T63">
+        <v>76</v>
+      </c>
+      <c r="U63">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="64" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>20</v>
+      </c>
+      <c r="B64" t="s">
+        <v>63</v>
+      </c>
+      <c r="C64">
+        <v>2026</v>
+      </c>
+      <c r="D64">
+        <v>267</v>
+      </c>
+      <c r="E64">
+        <v>0</v>
+      </c>
+      <c r="F64">
+        <v>0</v>
+      </c>
+      <c r="G64">
+        <v>0</v>
+      </c>
+      <c r="H64">
+        <v>2</v>
+      </c>
+      <c r="I64">
+        <v>3</v>
+      </c>
+      <c r="J64">
+        <v>10</v>
+      </c>
+      <c r="K64">
+        <v>267</v>
+      </c>
+      <c r="L64">
+        <v>20</v>
+      </c>
+      <c r="M64">
+        <v>24</v>
+      </c>
+      <c r="N64">
+        <v>40</v>
+      </c>
+      <c r="P64">
+        <v>43</v>
+      </c>
+      <c r="Q64">
+        <v>50</v>
+      </c>
+      <c r="T64">
+        <v>74</v>
+      </c>
+      <c r="U64">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="65" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>21</v>
+      </c>
+      <c r="B65" t="s">
+        <v>63</v>
+      </c>
+      <c r="C65">
+        <v>2026</v>
+      </c>
+      <c r="D65">
+        <v>124</v>
+      </c>
+      <c r="E65">
+        <v>0</v>
+      </c>
+      <c r="F65">
+        <v>0</v>
+      </c>
+      <c r="G65">
+        <v>0</v>
+      </c>
+      <c r="H65">
+        <v>3</v>
+      </c>
+      <c r="I65">
+        <v>4</v>
+      </c>
+      <c r="J65">
+        <v>11</v>
+      </c>
+      <c r="K65">
+        <v>124</v>
+      </c>
+      <c r="L65">
+        <v>22</v>
+      </c>
+      <c r="M65">
+        <v>26</v>
+      </c>
+      <c r="N65">
+        <v>32</v>
+      </c>
+      <c r="P65">
+        <v>34</v>
+      </c>
+      <c r="Q65">
+        <v>40</v>
+      </c>
+      <c r="T65">
+        <v>52</v>
+      </c>
+      <c r="U65">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="66" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>62</v>
+      </c>
+      <c r="B66" t="s">
+        <v>63</v>
+      </c>
+      <c r="C66">
+        <v>2026</v>
+      </c>
+      <c r="D66">
+        <v>53</v>
+      </c>
+      <c r="E66">
+        <v>0</v>
+      </c>
+      <c r="F66">
+        <v>0</v>
+      </c>
+      <c r="G66">
+        <v>0</v>
+      </c>
+      <c r="H66">
+        <v>0</v>
+      </c>
+      <c r="I66">
+        <v>1</v>
+      </c>
+      <c r="J66">
+        <v>3</v>
+      </c>
+      <c r="K66">
+        <v>53</v>
+      </c>
+      <c r="L66">
+        <v>3</v>
+      </c>
+      <c r="M66">
+        <v>3</v>
+      </c>
+      <c r="N66">
+        <v>5</v>
+      </c>
+      <c r="P66">
+        <v>5</v>
+      </c>
+      <c r="Q66">
+        <v>7</v>
+      </c>
+      <c r="T66">
+        <v>9</v>
+      </c>
+      <c r="U66">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="67" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>22</v>
+      </c>
+      <c r="B67" t="s">
+        <v>63</v>
+      </c>
+      <c r="C67">
+        <v>2026</v>
+      </c>
+      <c r="D67">
+        <v>60</v>
+      </c>
+      <c r="E67">
+        <v>0</v>
+      </c>
+      <c r="F67">
+        <v>0</v>
+      </c>
+      <c r="G67">
+        <v>0</v>
+      </c>
+      <c r="H67">
+        <v>1</v>
+      </c>
+      <c r="I67">
+        <v>3</v>
+      </c>
+      <c r="J67">
+        <v>6</v>
+      </c>
+      <c r="K67">
+        <v>60</v>
+      </c>
+      <c r="L67">
+        <v>9</v>
+      </c>
+      <c r="M67">
+        <v>10</v>
+      </c>
+      <c r="N67">
+        <v>15</v>
+      </c>
+      <c r="P67">
+        <v>16</v>
+      </c>
+      <c r="Q67">
+        <v>19</v>
+      </c>
+      <c r="T67">
+        <v>30</v>
+      </c>
+      <c r="U67">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="68" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>23</v>
+      </c>
+      <c r="B68" t="s">
+        <v>63</v>
+      </c>
+      <c r="C68">
+        <v>2026</v>
+      </c>
+      <c r="D68">
+        <v>140</v>
+      </c>
+      <c r="E68">
+        <v>1</v>
+      </c>
+      <c r="F68">
+        <v>1</v>
+      </c>
+      <c r="G68">
+        <v>5</v>
+      </c>
+      <c r="H68">
+        <v>10</v>
+      </c>
+      <c r="I68">
+        <v>12</v>
+      </c>
+      <c r="J68">
+        <v>23</v>
+      </c>
+      <c r="K68">
+        <v>140</v>
+      </c>
+      <c r="L68">
+        <v>35</v>
+      </c>
+      <c r="M68">
+        <v>37</v>
+      </c>
+      <c r="N68">
+        <v>46</v>
+      </c>
+      <c r="P68">
+        <v>48</v>
+      </c>
+      <c r="Q68">
+        <v>53</v>
+      </c>
+      <c r="T68">
+        <v>64</v>
+      </c>
+      <c r="U68">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="69" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>25</v>
+      </c>
+      <c r="B69" t="s">
+        <v>63</v>
+      </c>
+      <c r="C69">
+        <v>2026</v>
+      </c>
+      <c r="D69">
+        <v>67</v>
+      </c>
+      <c r="E69">
+        <v>0</v>
+      </c>
+      <c r="F69">
+        <v>0</v>
+      </c>
+      <c r="G69">
+        <v>0</v>
+      </c>
+      <c r="H69">
+        <v>0</v>
+      </c>
+      <c r="I69">
+        <v>1</v>
+      </c>
+      <c r="J69">
+        <v>6</v>
+      </c>
+      <c r="K69">
+        <v>67</v>
+      </c>
+      <c r="L69">
+        <v>13</v>
+      </c>
+      <c r="M69">
+        <v>16</v>
+      </c>
+      <c r="N69">
+        <v>24</v>
+      </c>
+      <c r="P69">
+        <v>24</v>
+      </c>
+      <c r="Q69">
+        <v>26</v>
+      </c>
+      <c r="T69">
+        <v>35</v>
+      </c>
+      <c r="U69">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="70" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>26</v>
+      </c>
+      <c r="B70" t="s">
+        <v>63</v>
+      </c>
+      <c r="C70">
+        <v>2026</v>
+      </c>
+      <c r="D70">
+        <v>51</v>
+      </c>
+      <c r="E70">
+        <v>0</v>
+      </c>
+      <c r="F70">
+        <v>0</v>
+      </c>
+      <c r="G70">
+        <v>0</v>
+      </c>
+      <c r="H70">
+        <v>0</v>
+      </c>
+      <c r="I70">
+        <v>0</v>
+      </c>
+      <c r="J70">
+        <v>1</v>
+      </c>
+      <c r="K70">
+        <v>51</v>
+      </c>
+      <c r="L70">
+        <v>1</v>
+      </c>
+      <c r="M70">
+        <v>4</v>
+      </c>
+      <c r="N70">
+        <v>4</v>
+      </c>
+      <c r="P70">
+        <v>5</v>
+      </c>
+      <c r="Q70">
+        <v>5</v>
+      </c>
+      <c r="T70">
+        <v>8</v>
+      </c>
+      <c r="U70">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="71" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>28</v>
+      </c>
+      <c r="B71" t="s">
+        <v>63</v>
+      </c>
+      <c r="C71">
+        <v>2026</v>
+      </c>
+      <c r="D71">
+        <v>159</v>
+      </c>
+      <c r="E71">
+        <v>0</v>
+      </c>
+      <c r="F71">
+        <v>2</v>
+      </c>
+      <c r="G71">
+        <v>9</v>
+      </c>
+      <c r="H71">
+        <v>17</v>
+      </c>
+      <c r="I71">
+        <v>19</v>
+      </c>
+      <c r="J71">
+        <v>38</v>
+      </c>
+      <c r="K71">
+        <v>159</v>
+      </c>
+      <c r="L71">
+        <v>56</v>
+      </c>
+      <c r="M71">
+        <v>61</v>
+      </c>
+      <c r="N71">
+        <v>81</v>
+      </c>
+      <c r="P71">
+        <v>86</v>
+      </c>
+      <c r="Q71">
+        <v>91</v>
+      </c>
+      <c r="T71">
+        <v>107</v>
+      </c>
+      <c r="U71">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="72" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>29</v>
+      </c>
+      <c r="B72" t="s">
+        <v>63</v>
+      </c>
+      <c r="C72">
+        <v>2026</v>
+      </c>
+      <c r="D72">
+        <v>57</v>
+      </c>
+      <c r="E72">
+        <v>0</v>
+      </c>
+      <c r="F72">
+        <v>0</v>
+      </c>
+      <c r="G72">
+        <v>0</v>
+      </c>
+      <c r="H72">
+        <v>0</v>
+      </c>
+      <c r="I72">
+        <v>0</v>
+      </c>
+      <c r="J72">
+        <v>0</v>
+      </c>
+      <c r="K72">
+        <v>57</v>
+      </c>
+      <c r="L72">
+        <v>7</v>
+      </c>
+      <c r="M72">
+        <v>9</v>
+      </c>
+      <c r="N72">
+        <v>14</v>
+      </c>
+      <c r="P72">
+        <v>16</v>
+      </c>
+      <c r="Q72">
+        <v>18</v>
+      </c>
+      <c r="T72">
+        <v>23</v>
+      </c>
+      <c r="U72">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="73" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>30</v>
+      </c>
+      <c r="B73" t="s">
+        <v>63</v>
+      </c>
+      <c r="C73">
+        <v>2026</v>
+      </c>
+      <c r="D73">
+        <v>102</v>
+      </c>
+      <c r="E73">
+        <v>0</v>
+      </c>
+      <c r="F73">
+        <v>0</v>
+      </c>
+      <c r="G73">
+        <v>0</v>
+      </c>
+      <c r="H73">
+        <v>5</v>
+      </c>
+      <c r="I73">
+        <v>7</v>
+      </c>
+      <c r="J73">
+        <v>16</v>
+      </c>
+      <c r="K73">
+        <v>102</v>
+      </c>
+      <c r="L73">
+        <v>24</v>
+      </c>
+      <c r="M73">
+        <v>29</v>
+      </c>
+      <c r="N73">
+        <v>44</v>
+      </c>
+      <c r="P73">
+        <v>46</v>
+      </c>
+      <c r="Q73">
+        <v>52</v>
+      </c>
+      <c r="T73">
+        <v>62</v>
+      </c>
+      <c r="U73">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="74" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>32</v>
+      </c>
+      <c r="B74" t="s">
+        <v>63</v>
+      </c>
+      <c r="C74">
+        <v>2026</v>
+      </c>
+      <c r="D74">
+        <v>32</v>
+      </c>
+      <c r="E74">
+        <v>0</v>
+      </c>
+      <c r="F74">
+        <v>0</v>
+      </c>
+      <c r="G74">
+        <v>0</v>
+      </c>
+      <c r="H74">
+        <v>0</v>
+      </c>
+      <c r="I74">
+        <v>0</v>
+      </c>
+      <c r="J74">
+        <v>1</v>
+      </c>
+      <c r="K74">
+        <v>32</v>
+      </c>
+      <c r="L74">
+        <v>2</v>
+      </c>
+      <c r="M74">
+        <v>3</v>
+      </c>
+      <c r="N74">
+        <v>4</v>
+      </c>
+      <c r="P74">
+        <v>6</v>
+      </c>
+      <c r="Q74">
+        <v>8</v>
+      </c>
+      <c r="T74">
+        <v>12</v>
+      </c>
+      <c r="U74">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="75" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>33</v>
+      </c>
+      <c r="B75" t="s">
+        <v>63</v>
+      </c>
+      <c r="C75">
+        <v>2026</v>
+      </c>
+      <c r="D75">
+        <v>79</v>
+      </c>
+      <c r="E75">
+        <v>0</v>
+      </c>
+      <c r="F75">
+        <v>1</v>
+      </c>
+      <c r="G75">
+        <v>4</v>
+      </c>
+      <c r="H75">
+        <v>6</v>
+      </c>
+      <c r="I75">
+        <v>8</v>
+      </c>
+      <c r="J75">
+        <v>13</v>
+      </c>
+      <c r="K75">
+        <v>79</v>
+      </c>
+      <c r="L75">
+        <v>17</v>
+      </c>
+      <c r="M75">
+        <v>21</v>
+      </c>
+      <c r="N75">
+        <v>35</v>
+      </c>
+      <c r="P75">
+        <v>38</v>
+      </c>
+      <c r="Q75">
+        <v>41</v>
+      </c>
+      <c r="T75">
+        <v>50</v>
+      </c>
+      <c r="U75">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="76" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>34</v>
+      </c>
+      <c r="B76" t="s">
+        <v>63</v>
+      </c>
+      <c r="C76">
+        <v>2026</v>
+      </c>
+      <c r="D76">
+        <v>231</v>
+      </c>
+      <c r="E76">
+        <v>0</v>
+      </c>
+      <c r="F76">
+        <v>0</v>
+      </c>
+      <c r="G76">
+        <v>2</v>
+      </c>
+      <c r="H76">
+        <v>4</v>
+      </c>
+      <c r="I76">
+        <v>5</v>
+      </c>
+      <c r="J76">
+        <v>15</v>
+      </c>
+      <c r="K76">
+        <v>231</v>
+      </c>
+      <c r="L76">
+        <v>23</v>
+      </c>
+      <c r="M76">
+        <v>26</v>
+      </c>
+      <c r="N76">
+        <v>45</v>
+      </c>
+      <c r="P76">
+        <v>48</v>
+      </c>
+      <c r="Q76">
+        <v>54</v>
+      </c>
+      <c r="T76">
+        <v>70</v>
+      </c>
+      <c r="U76">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="77" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>52</v>
+      </c>
+      <c r="B77" t="s">
+        <v>63</v>
+      </c>
+      <c r="C77">
+        <v>2026</v>
+      </c>
+      <c r="D77">
+        <v>15</v>
+      </c>
+      <c r="E77">
+        <v>0</v>
+      </c>
+      <c r="F77">
+        <v>0</v>
+      </c>
+      <c r="G77">
+        <v>0</v>
+      </c>
+      <c r="H77">
+        <v>0</v>
+      </c>
+      <c r="I77">
+        <v>0</v>
+      </c>
+      <c r="J77">
+        <v>0</v>
+      </c>
+      <c r="K77">
+        <v>15</v>
+      </c>
+      <c r="L77">
+        <v>0</v>
+      </c>
+      <c r="M77">
+        <v>0</v>
+      </c>
+      <c r="N77">
+        <v>1</v>
+      </c>
+      <c r="P77">
+        <v>1</v>
+      </c>
+      <c r="Q77">
+        <v>1</v>
+      </c>
+      <c r="T77">
+        <v>1</v>
+      </c>
+      <c r="U77">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>35</v>
+      </c>
+      <c r="B78" t="s">
+        <v>63</v>
+      </c>
+      <c r="C78">
+        <v>2026</v>
+      </c>
+      <c r="D78">
+        <v>18</v>
+      </c>
+      <c r="E78">
+        <v>0</v>
+      </c>
+      <c r="F78">
+        <v>0</v>
+      </c>
+      <c r="G78">
+        <v>0</v>
+      </c>
+      <c r="H78">
+        <v>0</v>
+      </c>
+      <c r="I78">
+        <v>0</v>
+      </c>
+      <c r="J78">
+        <v>0</v>
+      </c>
+      <c r="K78">
+        <v>18</v>
+      </c>
+      <c r="L78">
+        <v>2</v>
+      </c>
+      <c r="M78">
+        <v>2</v>
+      </c>
+      <c r="N78">
+        <v>3</v>
+      </c>
+      <c r="P78">
+        <v>3</v>
+      </c>
+      <c r="Q78">
+        <v>4</v>
+      </c>
+      <c r="T78">
+        <v>6</v>
+      </c>
+      <c r="U78">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="79" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>36</v>
+      </c>
+      <c r="B79" t="s">
+        <v>63</v>
+      </c>
+      <c r="C79">
+        <v>2026</v>
+      </c>
+      <c r="D79">
+        <v>40</v>
+      </c>
+      <c r="E79">
+        <v>0</v>
+      </c>
+      <c r="F79">
+        <v>0</v>
+      </c>
+      <c r="G79">
+        <v>0</v>
+      </c>
+      <c r="H79">
+        <v>0</v>
+      </c>
+      <c r="I79">
+        <v>0</v>
+      </c>
+      <c r="J79">
+        <v>1</v>
+      </c>
+      <c r="K79">
+        <v>40</v>
+      </c>
+      <c r="L79">
+        <v>3</v>
+      </c>
+      <c r="M79">
+        <v>3</v>
+      </c>
+      <c r="N79">
+        <v>5</v>
+      </c>
+      <c r="P79">
+        <v>6</v>
+      </c>
+      <c r="Q79">
+        <v>6</v>
+      </c>
+      <c r="T79">
+        <v>8</v>
+      </c>
+      <c r="U79">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="80" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>40</v>
+      </c>
+      <c r="B80" t="s">
+        <v>63</v>
+      </c>
+      <c r="C80">
+        <v>2026</v>
+      </c>
+      <c r="D80">
+        <v>101</v>
+      </c>
+      <c r="E80">
+        <v>0</v>
+      </c>
+      <c r="F80">
+        <v>0</v>
+      </c>
+      <c r="G80">
+        <v>1</v>
+      </c>
+      <c r="H80">
+        <v>3</v>
+      </c>
+      <c r="I80">
+        <v>4</v>
+      </c>
+      <c r="J80">
+        <v>6</v>
+      </c>
+      <c r="K80">
+        <v>101</v>
+      </c>
+      <c r="L80">
+        <v>9</v>
+      </c>
+      <c r="M80">
+        <v>11</v>
+      </c>
+      <c r="N80">
+        <v>19</v>
+      </c>
+      <c r="P80">
+        <v>24</v>
+      </c>
+      <c r="Q80">
+        <v>32</v>
+      </c>
+      <c r="T80">
+        <v>47</v>
+      </c>
+      <c r="U80">
+        <v>58</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:AA80" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:R1" numberStoredAsText="1"/>
+    <ignoredError sqref="T1:U1 A1:N1 P1:Q1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>